<commit_message>
add softAssertion and changes
</commit_message>
<xml_diff>
--- a/Automation-Framework/src/test/resources/testdata/TestData.xlsx
+++ b/Automation-Framework/src/test/resources/testdata/TestData.xlsx
@@ -4,19 +4,19 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016"/>
+    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="validLoginData" sheetId="1" r:id="rId1"/>
     <sheet name="inValidLoginData" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="empVerification" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="9">
   <si>
     <t>password</t>
   </si>
@@ -34,6 +34,15 @@
   </si>
   <si>
     <t>Tarun123@</t>
+  </si>
+  <si>
+    <t>emp_id</t>
+  </si>
+  <si>
+    <t>emp_name</t>
+  </si>
+  <si>
+    <t>sai</t>
   </si>
 </sst>
 </file>
@@ -425,9 +434,26 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
changes in testng.xml and run finaly
</commit_message>
<xml_diff>
--- a/Automation-Framework/src/test/resources/testdata/TestData.xlsx
+++ b/Automation-Framework/src/test/resources/testdata/TestData.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A529846F-1CD6-49BD-83A5-7E3C9B28BEA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" activeTab="2"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="validLoginData" sheetId="1" r:id="rId1"/>
@@ -42,14 +43,14 @@
     <t>emp_name</t>
   </si>
   <si>
-    <t>sai</t>
+    <t>Naveen</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -86,13 +87,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -130,7 +139,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -164,6 +173,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -198,9 +208,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -373,11 +384,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -385,7 +396,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -393,7 +404,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -407,11 +418,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -419,7 +430,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -433,11 +444,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -445,7 +456,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
changes in action and config and testdata
</commit_message>
<xml_diff>
--- a/Automation-Framework/src/test/resources/testdata/TestData.xlsx
+++ b/Automation-Framework/src/test/resources/testdata/TestData.xlsx
@@ -1,11 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A529846F-1CD6-49BD-83A5-7E3C9B28BEA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="validLoginData" sheetId="1" r:id="rId1"/>
@@ -43,14 +42,14 @@
     <t>emp_name</t>
   </si>
   <si>
-    <t>Naveen</t>
+    <t>sai</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -99,9 +98,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -139,7 +138,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -173,7 +172,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -208,10 +206,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -384,11 +381,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -396,7 +393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -404,7 +401,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -418,11 +415,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -430,7 +427,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -444,11 +441,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -456,7 +453,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2">
       <c r="A2">
         <v>2</v>
       </c>

</xml_diff>